<commit_message>
Fines controller was added and tested
</commit_message>
<xml_diff>
--- a/Utility/Security Desgin/LibraryUserCase.xlsx
+++ b/Utility/Security Desgin/LibraryUserCase.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>Entitiy</t>
   </si>
@@ -45,6 +45,9 @@
     <t>api/V1/Books</t>
   </si>
   <si>
+    <t>Done</t>
+  </si>
+  <si>
     <t xml:space="preserve">Get all books</t>
   </si>
   <si>
@@ -72,12 +75,12 @@
     <t>api/V1/Books/{BookName}</t>
   </si>
   <si>
+    <t xml:space="preserve">Get Single book</t>
+  </si>
+  <si>
     <t>User</t>
   </si>
   <si>
-    <t xml:space="preserve">Get Single book</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ability to adding user</t>
   </si>
   <si>
@@ -99,13 +102,19 @@
     <t xml:space="preserve">Get Single User</t>
   </si>
   <si>
+    <t xml:space="preserve">Get all User Fines</t>
+  </si>
+  <si>
+    <t>api/V1/User/{id}/Fines</t>
+  </si>
+  <si>
     <t>Reservations</t>
   </si>
   <si>
-    <t xml:space="preserve">Get all User Fines</t>
-  </si>
-  <si>
-    <t>api/V1/User/{id}/Fines</t>
+    <t xml:space="preserve">Complete Reservations</t>
+  </si>
+  <si>
+    <t>api/V1/Reservations/{id}/{status}</t>
   </si>
   <si>
     <t xml:space="preserve">Make Reservations</t>
@@ -117,21 +126,18 @@
     <t xml:space="preserve">Cancel Reservations</t>
   </si>
   <si>
-    <t>api/V1/Reservations/{id}/{status}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Get all Reservations</t>
   </si>
   <si>
+    <t xml:space="preserve">Get single Reservation</t>
+  </si>
+  <si>
+    <t>api/V1/Reservations/{id}</t>
+  </si>
+  <si>
     <t>Settings</t>
   </si>
   <si>
-    <t xml:space="preserve">Get single Reservation</t>
-  </si>
-  <si>
-    <t>api/V1/Reservations/{id}</t>
-  </si>
-  <si>
     <t xml:space="preserve">Update DefualtBorrrowDays</t>
   </si>
   <si>
@@ -159,10 +165,10 @@
     <t>api/V1/Fines/{id}</t>
   </si>
   <si>
-    <t xml:space="preserve">Get Payment Report</t>
-  </si>
-  <si>
-    <t>api/V1/Fines/Report</t>
+    <t xml:space="preserve">Get Payment Report Per User</t>
+  </si>
+  <si>
+    <t>api/V1/Fines/User/{UserId}/Report</t>
   </si>
   <si>
     <t>BorrowingRecords</t>
@@ -352,7 +358,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -406,15 +412,13 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left style="none"/>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="none"/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal style="none"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -450,19 +454,6 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left style="none"/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -493,6 +484,41 @@
     <border>
       <left style="none"/>
       <right style="none"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -527,7 +553,7 @@
     <xf fontId="7" fillId="11" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0"/>
     <xf fontId="7" fillId="12" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="7" fillId="12" borderId="0" numFmtId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -541,42 +567,53 @@
     <xf fontId="1" fillId="2" borderId="5" numFmtId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="7" fillId="10" borderId="5" numFmtId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="7" fillId="11" borderId="6" numFmtId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="2" fillId="13" borderId="7" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="1" fillId="2" borderId="8" numFmtId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="4" borderId="7" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="2" borderId="8" numFmtId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="7" fillId="10" borderId="8" numFmtId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="7" fillId="11" borderId="9" numFmtId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="3" fillId="4" borderId="10" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="2" fillId="3" borderId="4" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="2" borderId="9" numFmtId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="7" fillId="10" borderId="9" numFmtId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="7" fillId="11" borderId="10" numFmtId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="2" fillId="13" borderId="11" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="2" fillId="3" borderId="8" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="3" borderId="8" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="2" fillId="13" borderId="10" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="2" fillId="3" borderId="11" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="2" fillId="3" borderId="9" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="3" fillId="4" borderId="8" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="4" borderId="12" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="3" fillId="4" borderId="9" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="4" fillId="5" borderId="8" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="4" borderId="8" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="3" fillId="4" borderId="4" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="4" fillId="5" borderId="9" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="8" borderId="8" numFmtId="0" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="4" borderId="11" numFmtId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="8" borderId="9" numFmtId="0" xfId="7" applyFill="1" applyBorder="1"/>
-    <xf fontId="7" fillId="9" borderId="8" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="5" borderId="12" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="7" fillId="9" borderId="9" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="7" fillId="9" borderId="12" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="5" borderId="8" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="4" fillId="5" borderId="4" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="7" fillId="12" borderId="0" numFmtId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf fontId="4" fillId="5" borderId="11" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="7" fillId="12" borderId="9" numFmtId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="7" fillId="11" borderId="9" numFmtId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="13" numFmtId="0" xfId="7" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="8" borderId="8" numFmtId="0" xfId="7" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="8" borderId="8" numFmtId="0" xfId="7" applyFill="1" applyBorder="1"/>
+    <xf fontId="7" fillId="9" borderId="13" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="7" fillId="9" borderId="8" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="7" fillId="9" borderId="14" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="7" fillId="12" borderId="8" numFmtId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="7" fillId="11" borderId="8" numFmtId="0" xfId="10" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1135,453 +1172,485 @@
       <c r="D2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="7"/>
+      <c r="E2" s="7" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="12"/>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9" t="s">
+      <c r="A4" s="3"/>
+      <c r="B4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" ht="14.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="11" t="s">
+      <c r="D6" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" ht="14.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" ht="14.25">
+      <c r="A8" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="14"/>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="A9" s="12"/>
+      <c r="B9" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="12"/>
-    </row>
-    <row r="5" ht="14.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="11" t="s">
+      <c r="D9" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="14"/>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="A10" s="12"/>
+      <c r="B10" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="14"/>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="A11" s="12"/>
+      <c r="B11" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="14"/>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="A12" s="12"/>
+      <c r="B12" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="14"/>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="14"/>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="A14" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="18"/>
+      <c r="B15" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="18"/>
+      <c r="B16" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" ht="14.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="9" t="s">
+      <c r="D16" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17" s="18"/>
+      <c r="B17" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" s="19"/>
+      <c r="B18" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="21"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="14"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="22"/>
+      <c r="B20" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="14"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" s="22"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="14"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" s="23"/>
+      <c r="B22" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="14"/>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="A23" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="25"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="14"/>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" s="24"/>
+      <c r="B24" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" s="24"/>
+      <c r="B25" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" s="24"/>
+      <c r="B26" s="26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" s="24"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="14"/>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="A28" s="24"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="14"/>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="A29" s="24"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="14"/>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="A30" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E30" s="14"/>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="A31" s="27"/>
+      <c r="B31" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="14"/>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="A32" s="27"/>
+      <c r="B32" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E32" s="14"/>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="A33" s="27"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="14"/>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="A34" s="29"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="14"/>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="A35" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="E35" s="14"/>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="E36" s="14"/>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="A37" s="1"/>
+      <c r="B37" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="12"/>
-    </row>
-    <row r="7" ht="14.25">
-      <c r="A7" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="12"/>
-    </row>
-    <row r="8" ht="14.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="12"/>
-    </row>
-    <row r="9" ht="14.25">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="12"/>
-    </row>
-    <row r="10" ht="14.25">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="12"/>
-    </row>
-    <row r="11" ht="14.25">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="12"/>
-    </row>
-    <row r="12" ht="14.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" s="12"/>
-    </row>
-    <row r="13" ht="14.25">
-      <c r="A13" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="12"/>
-    </row>
-    <row r="14" ht="14.25">
-      <c r="A14" s="15"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="12"/>
-    </row>
-    <row r="15" ht="14.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="12"/>
-    </row>
-    <row r="16" ht="14.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="12"/>
-    </row>
-    <row r="17" ht="14.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" s="12"/>
-    </row>
-    <row r="18" ht="14.25">
-      <c r="A18" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="12"/>
-    </row>
-    <row r="19" ht="14.25">
-      <c r="A19" s="17"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="12"/>
-    </row>
-    <row r="20" ht="14.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="12"/>
-    </row>
-    <row r="21" ht="14.25">
-      <c r="A21" s="17"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="12"/>
-    </row>
-    <row r="22" ht="14.25">
-      <c r="A22" s="17"/>
-      <c r="B22" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="E22" s="12"/>
-    </row>
-    <row r="23" ht="14.25">
-      <c r="A23" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="12"/>
-    </row>
-    <row r="24" ht="14.25">
-      <c r="A24" s="19"/>
-      <c r="B24" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="E24" s="12"/>
-    </row>
-    <row r="25" ht="14.25">
-      <c r="A25" s="19"/>
-      <c r="B25" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="E25" s="12"/>
-    </row>
-    <row r="26" ht="14.25">
-      <c r="A26" s="19"/>
-      <c r="B26" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="E26" s="12"/>
-    </row>
-    <row r="27" ht="14.25">
-      <c r="A27" s="19"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="12"/>
-    </row>
-    <row r="28" ht="14.25">
-      <c r="A28" s="19"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="12"/>
-    </row>
-    <row r="29" ht="14.25">
-      <c r="A29" s="19"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="12"/>
-    </row>
-    <row r="30" ht="14.25">
-      <c r="A30" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B30" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C30" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E30" s="12"/>
-    </row>
-    <row r="31" ht="14.25">
-      <c r="A31" s="21"/>
-      <c r="B31" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="C31" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="E31" s="12"/>
-    </row>
-    <row r="32" ht="14.25">
-      <c r="A32" s="21"/>
-      <c r="B32" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="C32" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E32" s="12"/>
-    </row>
-    <row r="33" ht="14.25">
-      <c r="A33" s="21"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="12"/>
-    </row>
-    <row r="34" ht="14.25">
-      <c r="A34" s="23"/>
-      <c r="B34" s="22"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="12"/>
-    </row>
-    <row r="35" ht="14.25">
-      <c r="A35" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="B35" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="E35" s="12"/>
-    </row>
-    <row r="36" ht="14.25">
-      <c r="A36" s="24"/>
-      <c r="B36" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="26" t="s">
+      <c r="D37" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="E37" s="14"/>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="A38" s="1"/>
+      <c r="B38" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="E36" s="12"/>
-    </row>
-    <row r="37" ht="14.25">
-      <c r="A37" s="24"/>
-      <c r="B37" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="C37" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D37" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="E37" s="12"/>
-    </row>
-    <row r="38" ht="14.25">
-      <c r="A38" s="24"/>
-      <c r="B38" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="E38" s="12"/>
+      <c r="E38" s="14"/>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="24"/>
-      <c r="B39" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="E39" s="12"/>
+      <c r="A39" s="1"/>
+      <c r="B39" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="E39" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A7:A12"/>
-    <mergeCell ref="A13:A17"/>
-    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="A19:A22"/>
     <mergeCell ref="A23:A29"/>
     <mergeCell ref="A30:A34"/>
     <mergeCell ref="A35:A39"/>

</xml_diff>

<commit_message>
phone number was added and tested
</commit_message>
<xml_diff>
--- a/Utility/Security Desgin/LibraryUserCase.xlsx
+++ b/Utility/Security Desgin/LibraryUserCase.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>Entitiy</t>
   </si>
@@ -186,10 +186,10 @@
     <t>api/V1/BorrowingRecords</t>
   </si>
   <si>
-    <t xml:space="preserve">Cancel Borrowing</t>
-  </si>
-  <si>
-    <t>api/V1/BorrowingRecords/{id}/{Status}</t>
+    <t xml:space="preserve">Get Borrowing Record</t>
+  </si>
+  <si>
+    <t>api/V1/BorrowingRecords/{id}</t>
   </si>
   <si>
     <t xml:space="preserve">Phone number</t>
@@ -213,7 +213,10 @@
     <t>api/V1/Person/{PersonID}/PhoneNumbers/{Id}</t>
   </si>
   <si>
-    <t xml:space="preserve">Get all phone number with person info</t>
+    <t xml:space="preserve">GEt Phone numbers by  id</t>
+  </si>
+  <si>
+    <t>api/V1/PhoneNumbers/{id}</t>
   </si>
   <si>
     <t xml:space="preserve">GEt Phone numbers by person id</t>
@@ -358,7 +361,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="14">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -412,13 +415,13 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left/>
+      <left style="none"/>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -493,35 +496,11 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="none"/>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top style="none"/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -536,6 +515,19 @@
         <color auto="1"/>
       </top>
       <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal style="none"/>
     </border>
   </borders>
@@ -553,7 +545,7 @@
     <xf fontId="7" fillId="11" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0"/>
     <xf fontId="7" fillId="12" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="7" fillId="12" borderId="0" numFmtId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -604,12 +596,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="8" borderId="8" numFmtId="0" xfId="7" applyFill="1" applyBorder="1"/>
-    <xf fontId="0" fillId="8" borderId="8" numFmtId="0" xfId="7" applyFill="1" applyBorder="1"/>
     <xf fontId="7" fillId="9" borderId="13" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="7" fillId="9" borderId="8" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="7" fillId="9" borderId="14" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="7" fillId="9" borderId="12" numFmtId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="7" fillId="12" borderId="8" numFmtId="0" xfId="11" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1489,7 +1480,7 @@
     </row>
     <row r="26" ht="14.25">
       <c r="A26" s="24"/>
-      <c r="B26" s="26" t="s">
+      <c r="B26" s="25" t="s">
         <v>49</v>
       </c>
       <c r="C26" s="9" t="s">
@@ -1524,10 +1515,10 @@
       <c r="E29" s="14"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="27" t="s">
+      <c r="A30" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B30" s="28" t="s">
+      <c r="B30" s="27" t="s">
         <v>52</v>
       </c>
       <c r="C30" s="9" t="s">
@@ -1536,11 +1527,13 @@
       <c r="D30" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E30" s="14"/>
+      <c r="E30" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="27"/>
-      <c r="B31" s="28" t="s">
+      <c r="A31" s="26"/>
+      <c r="B31" s="27" t="s">
         <v>54</v>
       </c>
       <c r="C31" s="9" t="s">
@@ -1549,31 +1542,35 @@
       <c r="D31" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E31" s="14"/>
+      <c r="E31" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="27"/>
-      <c r="B32" s="28" t="s">
+      <c r="A32" s="26"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="14"/>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="A33" s="26"/>
+      <c r="B33" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="C32" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="10" t="s">
+      <c r="C33" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="E32" s="14"/>
-    </row>
-    <row r="33" ht="14.25">
-      <c r="A33" s="27"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="9"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="14"/>
+      <c r="E33" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="29"/>
-      <c r="B34" s="28"/>
+      <c r="A34" s="28"/>
+      <c r="B34" s="27"/>
       <c r="C34" s="9"/>
       <c r="D34" s="10"/>
       <c r="E34" s="14"/>
@@ -1582,66 +1579,66 @@
       <c r="A35" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B35" s="30" t="s">
+      <c r="B35" s="29" t="s">
         <v>59</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D35" s="31" t="s">
+      <c r="D35" s="30" t="s">
         <v>60</v>
       </c>
       <c r="E35" s="14"/>
     </row>
     <row r="36" ht="14.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="29" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D36" s="31" t="s">
+      <c r="D36" s="30" t="s">
         <v>62</v>
       </c>
       <c r="E36" s="14"/>
     </row>
     <row r="37" ht="14.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="30" t="s">
+      <c r="B37" s="29" t="s">
         <v>63</v>
       </c>
       <c r="C37" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="31" t="s">
+      <c r="D37" s="30" t="s">
         <v>64</v>
       </c>
       <c r="E37" s="14"/>
     </row>
     <row r="38" ht="14.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="30" t="s">
+      <c r="B38" s="29" t="s">
         <v>65</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D38" s="31" t="s">
-        <v>60</v>
+      <c r="D38" s="30" t="s">
+        <v>66</v>
       </c>
       <c r="E38" s="14"/>
     </row>
     <row r="39" ht="14.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="30" t="s">
-        <v>66</v>
+      <c r="B39" s="29" t="s">
+        <v>67</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D39" s="31" t="s">
-        <v>67</v>
+      <c r="D39" s="30" t="s">
+        <v>68</v>
       </c>
       <c r="E39" s="14"/>
     </row>

</xml_diff>

<commit_message>
User controller was added with testing
</commit_message>
<xml_diff>
--- a/Utility/Security Desgin/LibraryUserCase.xlsx
+++ b/Utility/Security Desgin/LibraryUserCase.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t>Entitiy</t>
   </si>
@@ -199,12 +199,6 @@
   </si>
   <si>
     <t>api/V1/PhoneNumbers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modifying phone number</t>
-  </si>
-  <si>
-    <t>api/V1/Person/{PersonID}/PhoneNumbers/{id}</t>
   </si>
   <si>
     <t xml:space="preserve">delete phone number</t>
@@ -1588,59 +1582,61 @@
       <c r="D35" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="E35" s="14"/>
+      <c r="E35" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="36" ht="14.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="E36" s="14"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="11"/>
     </row>
     <row r="37" ht="14.25">
       <c r="A37" s="1"/>
       <c r="B37" s="29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C37" s="9" t="s">
         <v>16</v>
       </c>
       <c r="D37" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="E37" s="14"/>
+        <v>62</v>
+      </c>
+      <c r="E37" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="38" ht="14.25">
       <c r="A38" s="1"/>
       <c r="B38" s="29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D38" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="E38" s="14"/>
+        <v>64</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="39" ht="14.25">
       <c r="A39" s="1"/>
       <c r="B39" s="29" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D39" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="E39" s="14"/>
+        <v>66</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Ending controllers and with testing cases
</commit_message>
<xml_diff>
--- a/Utility/Security Desgin/LibraryUserCase.xlsx
+++ b/Utility/Security Desgin/LibraryUserCase.xlsx
@@ -562,7 +562,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="3" borderId="8" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="2" fillId="13" borderId="10" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="2" fillId="3" borderId="11" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -580,6 +579,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="4" fillId="5" borderId="8" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="2" fillId="13" borderId="10" numFmtId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="4" fillId="5" borderId="4" numFmtId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1249,7 +1249,9 @@
       <c r="D8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="14"/>
+      <c r="E8" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="12"/>
@@ -1262,7 +1264,9 @@
       <c r="D9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="14"/>
+      <c r="E9" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" s="12"/>
@@ -1275,7 +1279,9 @@
       <c r="D10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="14"/>
+      <c r="E10" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" s="12"/>
@@ -1288,7 +1294,9 @@
       <c r="D11" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="14"/>
+      <c r="E11" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" s="12"/>
@@ -1301,10 +1309,12 @@
       <c r="D12" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="14"/>
+      <c r="E12" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="15"/>
+      <c r="A13" s="14"/>
       <c r="B13" s="13" t="s">
         <v>28</v>
       </c>
@@ -1314,13 +1324,15 @@
       <c r="D13" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="14"/>
+      <c r="E13" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="14" ht="14.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="16" t="s">
         <v>31</v>
       </c>
       <c r="C14" s="9"/>
@@ -1332,8 +1344,8 @@
       </c>
     </row>
     <row r="15" ht="14.25">
-      <c r="A15" s="18"/>
-      <c r="B15" s="17" t="s">
+      <c r="A15" s="17"/>
+      <c r="B15" s="16" t="s">
         <v>33</v>
       </c>
       <c r="C15" s="9" t="s">
@@ -1347,8 +1359,8 @@
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="18"/>
-      <c r="B16" s="17" t="s">
+      <c r="A16" s="17"/>
+      <c r="B16" s="16" t="s">
         <v>35</v>
       </c>
       <c r="C16" s="9" t="s">
@@ -1362,8 +1374,8 @@
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="18"/>
-      <c r="B17" s="17" t="s">
+      <c r="A17" s="17"/>
+      <c r="B17" s="16" t="s">
         <v>36</v>
       </c>
       <c r="C17" s="9" t="s">
@@ -1377,8 +1389,8 @@
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="19"/>
-      <c r="B18" s="17" t="s">
+      <c r="A18" s="18"/>
+      <c r="B18" s="16" t="s">
         <v>37</v>
       </c>
       <c r="C18" s="9" t="s">
@@ -1392,17 +1404,17 @@
       </c>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="20" t="s">
+      <c r="A19" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="21"/>
+      <c r="B19" s="20"/>
       <c r="C19" s="9"/>
       <c r="D19" s="10"/>
-      <c r="E19" s="14"/>
+      <c r="E19" s="21"/>
     </row>
     <row r="20" ht="14.25">
       <c r="A20" s="22"/>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>40</v>
       </c>
       <c r="C20" s="9" t="s">
@@ -1411,18 +1423,20 @@
       <c r="D20" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="E20" s="14"/>
+      <c r="E20" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="21" ht="14.25">
       <c r="A21" s="22"/>
-      <c r="B21" s="21"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="9"/>
       <c r="D21" s="10"/>
-      <c r="E21" s="14"/>
+      <c r="E21" s="21"/>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" s="23"/>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="20" t="s">
         <v>42</v>
       </c>
       <c r="C22" s="9" t="s">
@@ -1431,7 +1445,9 @@
       <c r="D22" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E22" s="14"/>
+      <c r="E22" s="11" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="23" ht="14.25">
       <c r="A23" s="24" t="s">
@@ -1440,7 +1456,7 @@
       <c r="B23" s="25"/>
       <c r="C23" s="9"/>
       <c r="D23" s="10"/>
-      <c r="E23" s="14"/>
+      <c r="E23" s="21"/>
     </row>
     <row r="24" ht="14.25">
       <c r="A24" s="24"/>
@@ -1492,21 +1508,21 @@
       <c r="B27" s="25"/>
       <c r="C27" s="9"/>
       <c r="D27" s="10"/>
-      <c r="E27" s="14"/>
+      <c r="E27" s="21"/>
     </row>
     <row r="28" ht="14.25">
       <c r="A28" s="24"/>
       <c r="B28" s="25"/>
       <c r="C28" s="9"/>
       <c r="D28" s="10"/>
-      <c r="E28" s="14"/>
+      <c r="E28" s="21"/>
     </row>
     <row r="29" ht="14.25">
       <c r="A29" s="24"/>
       <c r="B29" s="25"/>
       <c r="C29" s="9"/>
       <c r="D29" s="10"/>
-      <c r="E29" s="14"/>
+      <c r="E29" s="21"/>
     </row>
     <row r="30" ht="14.25">
       <c r="A30" s="26" t="s">
@@ -1545,7 +1561,7 @@
       <c r="B32" s="27"/>
       <c r="C32" s="9"/>
       <c r="D32" s="10"/>
-      <c r="E32" s="14"/>
+      <c r="E32" s="21"/>
     </row>
     <row r="33" ht="14.25">
       <c r="A33" s="26"/>
@@ -1567,7 +1583,7 @@
       <c r="B34" s="27"/>
       <c r="C34" s="9"/>
       <c r="D34" s="10"/>
-      <c r="E34" s="14"/>
+      <c r="E34" s="21"/>
     </row>
     <row r="35" ht="14.25">
       <c r="A35" s="1" t="s">

</xml_diff>